<commit_message>
Georgian template: editable statement + fix value overlap
Two fixes for template 4 (Georgian):

- The subtitle "კურსის წარმატებით დასრულებისთვის" is now an editable
  field (new optional "Statement" column; blank falls back to the
  default phrase), drawn by the app in BPG.

- Fixed dates/course overlapping leftover template text. The Georgian
  course and period values were baked into the artwork as live text PLUS
  a 0.5pt stroke (faux-bold) — a text layer and a vector layer. The old
  text-only redaction stripped neither reliably, so real data printed on
  top of the leftover. clean-templates.py now redacts both text and the
  stroke (PDF_REDACT_LINE_ART_REMOVE_IF_TOUCHED) over tight bands that
  sit just below the კურსი/პერიოდი labels, leaving the watermark intact.

Checked every field on all four templates renders cleanly with data that
differs from the artwork samples. certgen draws the statement; samples,
README and the e2e/render harnesses updated.
</commit_message>
<xml_diff>
--- a/app/samples/certificate-template-4-sample.xlsx
+++ b/app/samples/certificate-template-4-sample.xlsx
@@ -397,13 +397,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:F3"/>
   <cols>
     <col min="1" max="1" width="24.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
     <col min="3" max="3" width="24.83203125" customWidth="1"/>
     <col min="4" max="4" width="24.83203125" customWidth="1"/>
     <col min="5" max="5" width="24.83203125" customWidth="1"/>
+    <col min="6" max="6" width="24.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -422,6 +423,9 @@
       <c r="E1" t="str">
         <v>End Date</v>
       </c>
+      <c r="F1" t="str">
+        <v>Statement</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -439,6 +443,9 @@
       <c r="E2" t="str">
         <v>16.06.2026</v>
       </c>
+      <c r="F2" t="str">
+        <v>კურსის წარმატებით დასრულებისთვის</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -456,10 +463,13 @@
       <c r="E3" t="str">
         <v>01.07.2026</v>
       </c>
+      <c r="F3" t="str">
+        <v>კურსის წარმატებით დასრულებისთვის</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Georgian template: spreadsheet-driven date heading (პერიოდი/თარიღი)
The heading above the date range is baked into the artwork as "პერიოდი".
Add a per-row "Heading" column to the Georgian (kacourse) template so
users can override it (e.g. "თარიღი") straight from the spreadsheet,
instead of needing a separate template.

When a row supplies a heading other than the default, the baked word is
whited out and the chosen text is stamped in the same BPG caps font,
size, and position; blank cells keep the baked "პერიოდი". Sample rows
and the downloadable Georgian sheet demonstrate both values.
</commit_message>
<xml_diff>
--- a/app/samples/certificate-template-4-sample.xlsx
+++ b/app/samples/certificate-template-4-sample.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:G3"/>
   <cols>
     <col min="1" max="1" width="24.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -405,6 +405,7 @@
     <col min="4" max="4" width="24.83203125" customWidth="1"/>
     <col min="5" max="5" width="24.83203125" customWidth="1"/>
     <col min="6" max="6" width="24.83203125" customWidth="1"/>
+    <col min="7" max="7" width="24.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -426,6 +427,9 @@
       <c r="F1" t="str">
         <v>Statement</v>
       </c>
+      <c r="G1" t="str">
+        <v>Heading (პერიოდი/თარიღი)</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -446,6 +450,9 @@
       <c r="F2" t="str">
         <v>კურსის წარმატებით დასრულებისთვის</v>
       </c>
+      <c r="G2" t="str">
+        <v>პერიოდი</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -466,10 +473,13 @@
       <c r="F3" t="str">
         <v>კურსის წარმატებით დასრულებისთვის</v>
       </c>
+      <c r="G3" t="str">
+        <v>თარიღი</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>